<commit_message>
Create new region previews in the excel-sheets
</commit_message>
<xml_diff>
--- a/data/raw/Location.xlsx
+++ b/data/raw/Location.xlsx
@@ -1,26 +1,26 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11028"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10830"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/noraammann/Documents/Cloned_GitHub/daschland-scripts/data/raw/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/noemivillars-amberg/Documents/Customer_Projects/daschland-scripts/data/raw/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{036FE0E9-526D-4843-85F6-0A75FE7B2BC1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4D702E9D-4A79-7141-BA26-301827B3844B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="660" windowWidth="34560" windowHeight="20500" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="3620" yWindow="600" windowWidth="43720" windowHeight="24660" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="0" iterateDelta="1E-4"/>
+  <calcPr calcId="0"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="293" uniqueCount="232">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="296" uniqueCount="235">
   <si>
     <t>ID</t>
   </si>
@@ -716,6 +716,15 @@
   </si>
   <si>
     <t>https://www.wikidata.org/wiki/Q21</t>
+  </si>
+  <si>
+    <t>Region ID</t>
+  </si>
+  <si>
+    <t>R_008, R_009, R010</t>
+  </si>
+  <si>
+    <t>R011, R012</t>
   </si>
 </sst>
 </file>
@@ -823,7 +832,27 @@
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="2">
+  <dxfs count="3">
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="12"/>
+        <color rgb="FF000000"/>
+        <name val="Arial"/>
+        <family val="2"/>
+        <charset val="1"/>
+        <scheme val="none"/>
+      </font>
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
     <dxf>
       <font>
         <b val="0"/>
@@ -942,23 +971,24 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="Table1" displayName="Table1" ref="A1:K33" totalsRowShown="0">
-  <autoFilter ref="A1:K33" xr:uid="{00000000-0009-0000-0100-000001000000}"/>
-  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:J33">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="Table1" displayName="Table1" ref="A1:L33" totalsRowShown="0">
+  <autoFilter ref="A1:L33" xr:uid="{00000000-0009-0000-0100-000001000000}"/>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:K33">
     <sortCondition ref="A1:A33"/>
   </sortState>
-  <tableColumns count="11">
+  <tableColumns count="12">
     <tableColumn id="1" xr3:uid="{00000000-0010-0000-0000-000001000000}" name="ID"/>
     <tableColumn id="2" xr3:uid="{00000000-0010-0000-0000-000002000000}" name="Name"/>
     <tableColumn id="3" xr3:uid="{00000000-0010-0000-0000-000003000000}" name="Location Type List"/>
     <tableColumn id="4" xr3:uid="{00000000-0010-0000-0000-000004000000}" name="Geoname ID"/>
     <tableColumn id="5" xr3:uid="{00000000-0010-0000-0000-000005000000}" name="Image ID"/>
+    <tableColumn id="12" xr3:uid="{2BD6E00F-E1B9-4940-B657-7C672A29756B}" name="Region ID" dataDxfId="0"/>
     <tableColumn id="6" xr3:uid="{00000000-0010-0000-0000-000006000000}" name="Description EN"/>
     <tableColumn id="7" xr3:uid="{00000000-0010-0000-0000-000007000000}" name="Description DE"/>
     <tableColumn id="8" xr3:uid="{00000000-0010-0000-0000-000008000000}" name="Description FR"/>
     <tableColumn id="9" xr3:uid="{00000000-0010-0000-0000-000009000000}" name="Description IT"/>
-    <tableColumn id="10" xr3:uid="{00000000-0010-0000-0000-00000A000000}" name="Authorship Resource" dataDxfId="1"/>
-    <tableColumn id="11" xr3:uid="{1903091F-84E6-A345-8198-0CE678172009}" name="Wikidata Link" dataDxfId="0"/>
+    <tableColumn id="10" xr3:uid="{00000000-0010-0000-0000-00000A000000}" name="Authorship Resource" dataDxfId="2"/>
+    <tableColumn id="11" xr3:uid="{1903091F-84E6-A345-8198-0CE678172009}" name="Wikidata Link" dataDxfId="1"/>
   </tableColumns>
   <tableStyleInfo showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -1140,23 +1170,23 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:K37"/>
+  <dimension ref="A1:L37"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="12.6640625" defaultRowHeight="18" x14ac:dyDescent="0.15"/>
   <cols>
     <col min="1" max="1" width="12.6640625" style="1" customWidth="1"/>
     <col min="2" max="2" width="39.6640625" style="1" customWidth="1"/>
     <col min="4" max="4" width="12.1640625" style="1" customWidth="1"/>
-    <col min="5" max="5" width="25.6640625" style="1" customWidth="1"/>
-    <col min="6" max="6" width="66.33203125" style="1" customWidth="1"/>
-    <col min="7" max="7" width="72.6640625" style="1" customWidth="1"/>
-    <col min="8" max="8" width="80" style="1" customWidth="1"/>
-    <col min="9" max="9" width="76.33203125" style="1" customWidth="1"/>
-    <col min="10" max="10" width="42.5" style="1" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="17.6640625" style="1" bestFit="1" customWidth="1"/>
-    <col min="12" max="16384" width="12.6640625" style="1"/>
+    <col min="5" max="6" width="25.6640625" style="1" customWidth="1"/>
+    <col min="7" max="7" width="66.33203125" style="1" customWidth="1"/>
+    <col min="8" max="8" width="72.6640625" style="1" customWidth="1"/>
+    <col min="9" max="9" width="80" style="1" customWidth="1"/>
+    <col min="10" max="10" width="76.33203125" style="1" customWidth="1"/>
+    <col min="11" max="11" width="42.5" style="1" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="17.6640625" style="1" bestFit="1" customWidth="1"/>
+    <col min="13" max="16384" width="12.6640625" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" s="3" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="1" spans="1:12" s="3" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
@@ -1173,25 +1203,28 @@
         <v>4</v>
       </c>
       <c r="F1" s="2" t="s">
+        <v>232</v>
+      </c>
+      <c r="G1" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="2" t="s">
+      <c r="H1" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="2" t="s">
+      <c r="I1" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="2" t="s">
+      <c r="J1" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="3" t="s">
+      <c r="K1" s="3" t="s">
         <v>9</v>
       </c>
-      <c r="K1" s="3" t="s">
+      <c r="L1" s="3" t="s">
         <v>229</v>
       </c>
     </row>
-    <row r="2" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:12" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A2" s="4" t="s">
         <v>10</v>
       </c>
@@ -1203,23 +1236,24 @@
       </c>
       <c r="D2" s="4"/>
       <c r="E2" s="5"/>
-      <c r="F2" s="7" t="s">
+      <c r="F2" s="5"/>
+      <c r="G2" s="7" t="s">
         <v>13</v>
       </c>
-      <c r="G2" s="5" t="s">
+      <c r="H2" s="5" t="s">
         <v>14</v>
       </c>
-      <c r="H2" s="8" t="s">
+      <c r="I2" s="8" t="s">
         <v>15</v>
       </c>
-      <c r="I2" s="8" t="s">
+      <c r="J2" s="8" t="s">
         <v>16</v>
       </c>
-      <c r="J2" s="1" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="3" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="K2" s="1" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="3" spans="1:12" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A3" s="4" t="s">
         <v>18</v>
       </c>
@@ -1233,23 +1267,24 @@
       <c r="E3" s="5" t="s">
         <v>21</v>
       </c>
-      <c r="F3" s="7" t="s">
+      <c r="F3" s="5"/>
+      <c r="G3" s="7" t="s">
         <v>22</v>
       </c>
-      <c r="G3" s="5" t="s">
+      <c r="H3" s="5" t="s">
         <v>23</v>
       </c>
-      <c r="H3" s="8" t="s">
+      <c r="I3" s="8" t="s">
         <v>24</v>
       </c>
-      <c r="I3" s="8" t="s">
+      <c r="J3" s="8" t="s">
         <v>25</v>
       </c>
-      <c r="J3" s="1" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="4" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="K3" s="1" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="4" spans="1:12" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A4" s="4" t="s">
         <v>26</v>
       </c>
@@ -1263,23 +1298,24 @@
       <c r="E4" s="8" t="s">
         <v>28</v>
       </c>
-      <c r="F4" s="7" t="s">
+      <c r="F4" s="8"/>
+      <c r="G4" s="7" t="s">
         <v>29</v>
       </c>
-      <c r="G4" s="5" t="s">
+      <c r="H4" s="5" t="s">
         <v>30</v>
       </c>
-      <c r="H4" s="8" t="s">
+      <c r="I4" s="8" t="s">
         <v>31</v>
       </c>
-      <c r="I4" s="8" t="s">
+      <c r="J4" s="8" t="s">
         <v>32</v>
       </c>
-      <c r="J4" s="1" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="5" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="K4" s="1" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="5" spans="1:12" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A5" s="4" t="s">
         <v>33</v>
       </c>
@@ -1293,23 +1329,26 @@
       <c r="E5" s="8" t="s">
         <v>35</v>
       </c>
-      <c r="F5" s="7" t="s">
+      <c r="F5" s="8" t="s">
+        <v>233</v>
+      </c>
+      <c r="G5" s="7" t="s">
         <v>36</v>
       </c>
-      <c r="G5" s="5" t="s">
+      <c r="H5" s="5" t="s">
         <v>37</v>
       </c>
-      <c r="H5" s="8" t="s">
+      <c r="I5" s="8" t="s">
         <v>38</v>
       </c>
-      <c r="I5" s="8" t="s">
+      <c r="J5" s="8" t="s">
         <v>39</v>
       </c>
-      <c r="J5" s="1" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="6" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="K5" s="1" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="6" spans="1:12" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A6" s="4" t="s">
         <v>40</v>
       </c>
@@ -1321,23 +1360,24 @@
       </c>
       <c r="D6" s="4"/>
       <c r="E6" s="5"/>
-      <c r="F6" s="7" t="s">
+      <c r="F6" s="5"/>
+      <c r="G6" s="7" t="s">
         <v>42</v>
       </c>
-      <c r="G6" s="5" t="s">
+      <c r="H6" s="5" t="s">
         <v>43</v>
       </c>
-      <c r="H6" s="8" t="s">
+      <c r="I6" s="8" t="s">
         <v>44</v>
       </c>
-      <c r="I6" s="8" t="s">
+      <c r="J6" s="8" t="s">
         <v>45</v>
       </c>
-      <c r="J6" s="1" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="7" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="K6" s="1" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="7" spans="1:12" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A7" s="4" t="s">
         <v>46</v>
       </c>
@@ -1349,23 +1389,24 @@
       </c>
       <c r="D7" s="4"/>
       <c r="E7" s="5"/>
-      <c r="F7" s="7" t="s">
+      <c r="F7" s="5"/>
+      <c r="G7" s="7" t="s">
         <v>48</v>
       </c>
-      <c r="G7" s="5" t="s">
+      <c r="H7" s="5" t="s">
         <v>49</v>
       </c>
-      <c r="H7" s="8" t="s">
+      <c r="I7" s="8" t="s">
         <v>50</v>
       </c>
-      <c r="I7" s="8" t="s">
+      <c r="J7" s="8" t="s">
         <v>51</v>
       </c>
-      <c r="J7" s="1" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="8" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="K7" s="1" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="8" spans="1:12" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A8" s="4" t="s">
         <v>52</v>
       </c>
@@ -1379,23 +1420,24 @@
       <c r="E8" s="8" t="s">
         <v>54</v>
       </c>
-      <c r="F8" s="7" t="s">
+      <c r="F8" s="8"/>
+      <c r="G8" s="7" t="s">
         <v>55</v>
       </c>
-      <c r="G8" s="5" t="s">
+      <c r="H8" s="5" t="s">
         <v>56</v>
       </c>
-      <c r="H8" s="8" t="s">
+      <c r="I8" s="8" t="s">
         <v>57</v>
       </c>
-      <c r="I8" s="8" t="s">
+      <c r="J8" s="8" t="s">
         <v>58</v>
       </c>
-      <c r="J8" s="1" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="9" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="K8" s="1" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="9" spans="1:12" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A9" s="4" t="s">
         <v>59</v>
       </c>
@@ -1409,23 +1451,24 @@
       <c r="E9" s="5" t="s">
         <v>61</v>
       </c>
-      <c r="F9" s="7" t="s">
+      <c r="F9" s="5"/>
+      <c r="G9" s="7" t="s">
         <v>62</v>
       </c>
-      <c r="G9" s="5" t="s">
+      <c r="H9" s="5" t="s">
         <v>63</v>
       </c>
-      <c r="H9" s="8" t="s">
+      <c r="I9" s="8" t="s">
         <v>64</v>
       </c>
-      <c r="I9" s="8" t="s">
+      <c r="J9" s="8" t="s">
         <v>65</v>
       </c>
-      <c r="J9" s="1" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="10" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="K9" s="1" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="10" spans="1:12" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A10" s="4" t="s">
         <v>66</v>
       </c>
@@ -1439,26 +1482,27 @@
         <v>2640729</v>
       </c>
       <c r="E10" s="5"/>
-      <c r="F10" s="7" t="s">
+      <c r="F10" s="5"/>
+      <c r="G10" s="7" t="s">
         <v>68</v>
       </c>
-      <c r="G10" s="5" t="s">
+      <c r="H10" s="5" t="s">
         <v>69</v>
       </c>
-      <c r="H10" s="8" t="s">
+      <c r="I10" s="8" t="s">
         <v>70</v>
       </c>
-      <c r="I10" s="8" t="s">
+      <c r="J10" s="8" t="s">
         <v>71</v>
       </c>
-      <c r="J10" s="1" t="s">
-        <v>17</v>
-      </c>
       <c r="K10" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="L10" s="1" t="s">
         <v>230</v>
       </c>
     </row>
-    <row r="11" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:12" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A11" s="4" t="s">
         <v>72</v>
       </c>
@@ -1472,26 +1516,27 @@
         <v>6269131</v>
       </c>
       <c r="E11" s="5"/>
-      <c r="F11" s="7" t="s">
+      <c r="F11" s="5"/>
+      <c r="G11" s="7" t="s">
         <v>74</v>
       </c>
-      <c r="G11" s="5" t="s">
+      <c r="H11" s="5" t="s">
         <v>75</v>
       </c>
-      <c r="H11" s="8" t="s">
+      <c r="I11" s="8" t="s">
         <v>76</v>
       </c>
-      <c r="I11" s="8" t="s">
+      <c r="J11" s="8" t="s">
         <v>77</v>
       </c>
-      <c r="J11" s="1" t="s">
-        <v>17</v>
-      </c>
       <c r="K11" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="L11" s="1" t="s">
         <v>231</v>
       </c>
     </row>
-    <row r="12" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:12" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A12" s="4" t="s">
         <v>78</v>
       </c>
@@ -1505,23 +1550,24 @@
       <c r="E12" s="5" t="s">
         <v>80</v>
       </c>
-      <c r="F12" s="7" t="s">
+      <c r="F12" s="5"/>
+      <c r="G12" s="7" t="s">
         <v>81</v>
       </c>
-      <c r="G12" s="5" t="s">
+      <c r="H12" s="5" t="s">
         <v>82</v>
       </c>
-      <c r="H12" s="8" t="s">
+      <c r="I12" s="8" t="s">
         <v>83</v>
       </c>
-      <c r="I12" s="8" t="s">
+      <c r="J12" s="8" t="s">
         <v>84</v>
       </c>
-      <c r="J12" s="1" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="13" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="K12" s="1" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="13" spans="1:12" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A13" s="4" t="s">
         <v>85</v>
       </c>
@@ -1535,23 +1581,24 @@
       <c r="E13" s="8" t="s">
         <v>87</v>
       </c>
-      <c r="F13" s="7" t="s">
+      <c r="F13" s="8"/>
+      <c r="G13" s="7" t="s">
         <v>88</v>
       </c>
-      <c r="G13" s="5" t="s">
+      <c r="H13" s="5" t="s">
         <v>89</v>
       </c>
-      <c r="H13" s="8" t="s">
+      <c r="I13" s="8" t="s">
         <v>90</v>
       </c>
-      <c r="I13" s="8" t="s">
+      <c r="J13" s="8" t="s">
         <v>91</v>
       </c>
-      <c r="J13" s="1" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="14" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="K13" s="1" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="14" spans="1:12" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A14" s="4" t="s">
         <v>92</v>
       </c>
@@ -1565,23 +1612,24 @@
       <c r="E14" s="5" t="s">
         <v>94</v>
       </c>
-      <c r="F14" s="7" t="s">
+      <c r="F14" s="5"/>
+      <c r="G14" s="7" t="s">
         <v>95</v>
       </c>
-      <c r="G14" s="5" t="s">
+      <c r="H14" s="5" t="s">
         <v>96</v>
       </c>
-      <c r="H14" s="8" t="s">
+      <c r="I14" s="8" t="s">
         <v>97</v>
       </c>
-      <c r="I14" s="8" t="s">
+      <c r="J14" s="8" t="s">
         <v>98</v>
       </c>
-      <c r="J14" s="1" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="15" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="K14" s="1" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="15" spans="1:12" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A15" s="4" t="s">
         <v>99</v>
       </c>
@@ -1595,23 +1643,24 @@
       <c r="E15" s="8" t="s">
         <v>101</v>
       </c>
-      <c r="F15" s="7" t="s">
+      <c r="F15" s="8"/>
+      <c r="G15" s="7" t="s">
         <v>102</v>
       </c>
-      <c r="G15" s="5" t="s">
+      <c r="H15" s="5" t="s">
         <v>103</v>
       </c>
-      <c r="H15" s="8" t="s">
+      <c r="I15" s="8" t="s">
         <v>104</v>
       </c>
-      <c r="I15" s="8" t="s">
+      <c r="J15" s="8" t="s">
         <v>105</v>
       </c>
-      <c r="J15" s="1" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="16" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="K15" s="1" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="16" spans="1:12" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A16" s="4" t="s">
         <v>106</v>
       </c>
@@ -1623,23 +1672,24 @@
       </c>
       <c r="D16" s="6"/>
       <c r="E16" s="5"/>
-      <c r="F16" s="7" t="s">
+      <c r="F16" s="5"/>
+      <c r="G16" s="7" t="s">
         <v>108</v>
       </c>
-      <c r="G16" s="5" t="s">
+      <c r="H16" s="5" t="s">
         <v>109</v>
       </c>
-      <c r="H16" s="8" t="s">
+      <c r="I16" s="8" t="s">
         <v>110</v>
       </c>
-      <c r="I16" s="8" t="s">
+      <c r="J16" s="8" t="s">
         <v>111</v>
       </c>
-      <c r="J16" s="1" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="17" spans="1:10" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="K16" s="1" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="17" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A17" s="4" t="s">
         <v>112</v>
       </c>
@@ -1653,23 +1703,24 @@
       <c r="E17" s="8" t="s">
         <v>114</v>
       </c>
-      <c r="F17" s="7" t="s">
+      <c r="F17" s="8"/>
+      <c r="G17" s="7" t="s">
         <v>115</v>
       </c>
-      <c r="G17" s="5" t="s">
+      <c r="H17" s="5" t="s">
         <v>116</v>
       </c>
-      <c r="H17" s="8" t="s">
+      <c r="I17" s="8" t="s">
         <v>117</v>
       </c>
-      <c r="I17" s="8" t="s">
+      <c r="J17" s="8" t="s">
         <v>118</v>
       </c>
-      <c r="J17" s="1" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="18" spans="1:10" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="K17" s="1" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="18" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A18" s="4" t="s">
         <v>119</v>
       </c>
@@ -1683,23 +1734,24 @@
       <c r="E18" s="8" t="s">
         <v>121</v>
       </c>
-      <c r="F18" s="7" t="s">
+      <c r="F18" s="8"/>
+      <c r="G18" s="7" t="s">
         <v>122</v>
       </c>
-      <c r="G18" s="5" t="s">
+      <c r="H18" s="5" t="s">
         <v>123</v>
       </c>
-      <c r="H18" s="8" t="s">
+      <c r="I18" s="8" t="s">
         <v>124</v>
       </c>
-      <c r="I18" s="8" t="s">
+      <c r="J18" s="8" t="s">
         <v>125</v>
       </c>
-      <c r="J18" s="1" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="19" spans="1:10" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="K18" s="1" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="19" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A19" s="4" t="s">
         <v>126</v>
       </c>
@@ -1713,23 +1765,24 @@
       <c r="E19" s="8" t="s">
         <v>128</v>
       </c>
-      <c r="F19" s="7" t="s">
+      <c r="F19" s="8"/>
+      <c r="G19" s="7" t="s">
         <v>129</v>
       </c>
-      <c r="G19" s="5" t="s">
+      <c r="H19" s="5" t="s">
         <v>130</v>
       </c>
-      <c r="H19" s="8" t="s">
+      <c r="I19" s="8" t="s">
         <v>131</v>
       </c>
-      <c r="I19" s="8" t="s">
+      <c r="J19" s="8" t="s">
         <v>132</v>
       </c>
-      <c r="J19" s="1" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="20" spans="1:10" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="K19" s="1" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="20" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A20" s="4" t="s">
         <v>133</v>
       </c>
@@ -1743,23 +1796,24 @@
       <c r="E20" s="5" t="s">
         <v>135</v>
       </c>
-      <c r="F20" s="7" t="s">
+      <c r="F20" s="5"/>
+      <c r="G20" s="7" t="s">
         <v>136</v>
       </c>
-      <c r="G20" s="5" t="s">
+      <c r="H20" s="5" t="s">
         <v>137</v>
       </c>
-      <c r="H20" s="8" t="s">
+      <c r="I20" s="8" t="s">
         <v>138</v>
       </c>
-      <c r="I20" s="8" t="s">
+      <c r="J20" s="8" t="s">
         <v>139</v>
       </c>
-      <c r="J20" s="1" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="21" spans="1:10" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="K20" s="1" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="21" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A21" s="4" t="s">
         <v>140</v>
       </c>
@@ -1773,23 +1827,24 @@
       <c r="E21" s="5" t="s">
         <v>142</v>
       </c>
-      <c r="F21" s="7" t="s">
+      <c r="F21" s="5"/>
+      <c r="G21" s="7" t="s">
         <v>143</v>
       </c>
-      <c r="G21" s="5" t="s">
+      <c r="H21" s="5" t="s">
         <v>144</v>
       </c>
-      <c r="H21" s="8" t="s">
+      <c r="I21" s="8" t="s">
         <v>145</v>
       </c>
-      <c r="I21" s="8" t="s">
+      <c r="J21" s="8" t="s">
         <v>146</v>
       </c>
-      <c r="J21" s="1" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="22" spans="1:10" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="K21" s="1" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="22" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A22" s="4" t="s">
         <v>147</v>
       </c>
@@ -1803,23 +1858,26 @@
       <c r="E22" s="8" t="s">
         <v>149</v>
       </c>
-      <c r="F22" s="7" t="s">
+      <c r="F22" s="8" t="s">
+        <v>234</v>
+      </c>
+      <c r="G22" s="7" t="s">
         <v>150</v>
       </c>
-      <c r="G22" s="5" t="s">
+      <c r="H22" s="5" t="s">
         <v>151</v>
       </c>
-      <c r="H22" s="8" t="s">
+      <c r="I22" s="8" t="s">
         <v>152</v>
       </c>
-      <c r="I22" s="8" t="s">
+      <c r="J22" s="8" t="s">
         <v>153</v>
       </c>
-      <c r="J22" s="1" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="23" spans="1:10" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="K22" s="1" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="23" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A23" s="4" t="s">
         <v>154</v>
       </c>
@@ -1833,23 +1891,24 @@
       <c r="E23" s="5" t="s">
         <v>156</v>
       </c>
-      <c r="F23" s="7" t="s">
+      <c r="F23" s="5"/>
+      <c r="G23" s="7" t="s">
         <v>157</v>
       </c>
-      <c r="G23" s="5" t="s">
+      <c r="H23" s="5" t="s">
         <v>158</v>
       </c>
-      <c r="H23" s="8" t="s">
+      <c r="I23" s="8" t="s">
         <v>159</v>
       </c>
-      <c r="I23" s="8" t="s">
+      <c r="J23" s="8" t="s">
         <v>160</v>
       </c>
-      <c r="J23" s="1" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="24" spans="1:10" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="K23" s="1" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="24" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A24" s="4" t="s">
         <v>161</v>
       </c>
@@ -1863,23 +1922,24 @@
       <c r="E24" s="8" t="s">
         <v>163</v>
       </c>
-      <c r="F24" s="7" t="s">
+      <c r="F24" s="8"/>
+      <c r="G24" s="7" t="s">
         <v>164</v>
       </c>
-      <c r="G24" s="5" t="s">
+      <c r="H24" s="5" t="s">
         <v>165</v>
       </c>
-      <c r="H24" s="8" t="s">
+      <c r="I24" s="8" t="s">
         <v>166</v>
       </c>
-      <c r="I24" s="8" t="s">
+      <c r="J24" s="8" t="s">
         <v>167</v>
       </c>
-      <c r="J24" s="1" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="25" spans="1:10" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="K24" s="1" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="25" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A25" s="4" t="s">
         <v>168</v>
       </c>
@@ -1893,23 +1953,24 @@
       <c r="E25" s="5" t="s">
         <v>170</v>
       </c>
-      <c r="F25" s="7" t="s">
+      <c r="F25" s="5"/>
+      <c r="G25" s="7" t="s">
         <v>171</v>
       </c>
-      <c r="G25" s="5" t="s">
+      <c r="H25" s="5" t="s">
         <v>172</v>
       </c>
-      <c r="H25" s="8" t="s">
+      <c r="I25" s="8" t="s">
         <v>173</v>
       </c>
-      <c r="I25" s="8" t="s">
+      <c r="J25" s="8" t="s">
         <v>174</v>
       </c>
-      <c r="J25" s="1" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="26" spans="1:10" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="K25" s="1" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="26" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A26" s="4" t="s">
         <v>175</v>
       </c>
@@ -1923,23 +1984,24 @@
       <c r="E26" s="5" t="s">
         <v>177</v>
       </c>
-      <c r="F26" s="7" t="s">
+      <c r="F26" s="5"/>
+      <c r="G26" s="7" t="s">
         <v>178</v>
       </c>
-      <c r="G26" s="5" t="s">
+      <c r="H26" s="5" t="s">
         <v>179</v>
       </c>
-      <c r="H26" s="8" t="s">
+      <c r="I26" s="8" t="s">
         <v>180</v>
       </c>
-      <c r="I26" s="8" t="s">
+      <c r="J26" s="8" t="s">
         <v>181</v>
       </c>
-      <c r="J26" s="1" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="27" spans="1:10" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="K26" s="1" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="27" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A27" s="4" t="s">
         <v>182</v>
       </c>
@@ -1953,23 +2015,24 @@
       <c r="E27" s="8" t="s">
         <v>184</v>
       </c>
-      <c r="F27" s="7" t="s">
+      <c r="F27" s="8"/>
+      <c r="G27" s="7" t="s">
         <v>185</v>
       </c>
-      <c r="G27" s="5" t="s">
+      <c r="H27" s="5" t="s">
         <v>186</v>
       </c>
-      <c r="H27" s="8" t="s">
+      <c r="I27" s="8" t="s">
         <v>187</v>
       </c>
-      <c r="I27" s="8" t="s">
+      <c r="J27" s="8" t="s">
         <v>188</v>
       </c>
-      <c r="J27" s="1" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="28" spans="1:10" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="K27" s="1" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="28" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A28" s="4" t="s">
         <v>189</v>
       </c>
@@ -1983,23 +2046,24 @@
       <c r="E28" s="8" t="s">
         <v>191</v>
       </c>
-      <c r="F28" s="7" t="s">
+      <c r="F28" s="8"/>
+      <c r="G28" s="7" t="s">
         <v>192</v>
       </c>
-      <c r="G28" s="5" t="s">
+      <c r="H28" s="5" t="s">
         <v>193</v>
       </c>
-      <c r="H28" s="8" t="s">
+      <c r="I28" s="8" t="s">
         <v>194</v>
       </c>
-      <c r="I28" s="8" t="s">
+      <c r="J28" s="8" t="s">
         <v>195</v>
       </c>
-      <c r="J28" s="1" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="29" spans="1:10" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="K28" s="1" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="29" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A29" s="4" t="s">
         <v>196</v>
       </c>
@@ -2013,23 +2077,24 @@
       <c r="E29" s="5" t="s">
         <v>198</v>
       </c>
-      <c r="F29" s="7" t="s">
+      <c r="F29" s="5"/>
+      <c r="G29" s="7" t="s">
         <v>199</v>
       </c>
-      <c r="G29" s="5" t="s">
+      <c r="H29" s="5" t="s">
         <v>200</v>
       </c>
-      <c r="H29" s="8" t="s">
+      <c r="I29" s="8" t="s">
         <v>201</v>
       </c>
-      <c r="I29" s="8" t="s">
+      <c r="J29" s="8" t="s">
         <v>202</v>
       </c>
-      <c r="J29" s="1" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="30" spans="1:10" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="K29" s="1" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="30" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A30" s="4" t="s">
         <v>203</v>
       </c>
@@ -2043,23 +2108,24 @@
       <c r="E30" s="5" t="s">
         <v>205</v>
       </c>
-      <c r="F30" s="7" t="s">
+      <c r="F30" s="5"/>
+      <c r="G30" s="7" t="s">
         <v>206</v>
       </c>
-      <c r="G30" s="5" t="s">
+      <c r="H30" s="5" t="s">
         <v>207</v>
       </c>
-      <c r="H30" s="8" t="s">
+      <c r="I30" s="8" t="s">
         <v>208</v>
       </c>
-      <c r="I30" s="8" t="s">
+      <c r="J30" s="8" t="s">
         <v>209</v>
       </c>
-      <c r="J30" s="1" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="31" spans="1:10" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="K30" s="1" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="31" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A31" s="4" t="s">
         <v>210</v>
       </c>
@@ -2073,23 +2139,24 @@
       <c r="E31" s="5" t="s">
         <v>212</v>
       </c>
-      <c r="F31" s="7" t="s">
+      <c r="F31" s="5"/>
+      <c r="G31" s="7" t="s">
         <v>213</v>
       </c>
-      <c r="G31" s="5" t="s">
+      <c r="H31" s="5" t="s">
         <v>214</v>
       </c>
-      <c r="H31" s="8" t="s">
+      <c r="I31" s="8" t="s">
         <v>215</v>
       </c>
-      <c r="I31" s="8" t="s">
+      <c r="J31" s="8" t="s">
         <v>216</v>
       </c>
-      <c r="J31" s="1" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="32" spans="1:10" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="K31" s="1" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="32" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A32" s="4" t="s">
         <v>217</v>
       </c>
@@ -2101,23 +2168,24 @@
       </c>
       <c r="D32" s="6"/>
       <c r="E32" s="5"/>
-      <c r="F32" s="7" t="s">
+      <c r="F32" s="5"/>
+      <c r="G32" s="7" t="s">
         <v>219</v>
       </c>
-      <c r="G32" s="5" t="s">
+      <c r="H32" s="5" t="s">
         <v>220</v>
       </c>
-      <c r="H32" s="8" t="s">
+      <c r="I32" s="8" t="s">
         <v>221</v>
       </c>
-      <c r="I32" s="8" t="s">
+      <c r="J32" s="8" t="s">
         <v>222</v>
       </c>
-      <c r="J32" s="1" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="33" spans="1:10" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="K32" s="1" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="33" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A33" s="4" t="s">
         <v>223</v>
       </c>
@@ -2129,32 +2197,33 @@
       </c>
       <c r="D33" s="6"/>
       <c r="E33" s="5"/>
-      <c r="F33" s="7" t="s">
+      <c r="F33" s="5"/>
+      <c r="G33" s="7" t="s">
         <v>225</v>
       </c>
-      <c r="G33" s="5" t="s">
+      <c r="H33" s="5" t="s">
         <v>226</v>
       </c>
-      <c r="H33" s="8" t="s">
+      <c r="I33" s="8" t="s">
         <v>227</v>
       </c>
-      <c r="I33" s="8" t="s">
+      <c r="J33" s="8" t="s">
         <v>228</v>
       </c>
-      <c r="J33" s="1" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="34" spans="1:10" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="K33" s="1" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="34" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="B34" s="10"/>
     </row>
-    <row r="35" spans="1:10" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="35" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="B35" s="10"/>
     </row>
-    <row r="36" spans="1:10" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="36" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="B36" s="10"/>
     </row>
-    <row r="37" spans="1:10" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="37" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="B37" s="10"/>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
data update with new columns for coordinates
</commit_message>
<xml_diff>
--- a/data/raw/Location.xlsx
+++ b/data/raw/Location.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10830"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11011"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/noemivillars-amberg/Documents/Customer_Projects/daschland-scripts/data/raw/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B56144AB-D8DD-4B42-9FD6-EA3A789C598A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{58AC83C3-642F-5741-B88D-B91CA9E1BD10}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="3620" yWindow="600" windowWidth="43720" windowHeight="24660" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="10680" yWindow="10660" windowWidth="64460" windowHeight="24660" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="296" uniqueCount="235">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="298" uniqueCount="237">
   <si>
     <t>ID</t>
   </si>
@@ -725,6 +725,12 @@
   </si>
   <si>
     <t>R_008, R_009, R_010</t>
+  </si>
+  <si>
+    <t>Coordinates Longitude</t>
+  </si>
+  <si>
+    <t>Coordinates Latitude</t>
   </si>
 </sst>
 </file>
@@ -832,7 +838,7 @@
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="3">
+  <dxfs count="5">
     <dxf>
       <font>
         <b val="0"/>
@@ -888,6 +894,46 @@
         <scheme val="none"/>
       </font>
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="12"/>
+        <color rgb="FF000000"/>
+        <name val="Arial"/>
+        <family val="2"/>
+        <charset val="1"/>
+        <scheme val="none"/>
+      </font>
+      <alignment horizontal="left" vertical="top" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="12"/>
+        <color rgb="FF000000"/>
+        <name val="Arial"/>
+        <family val="2"/>
+        <charset val="1"/>
+        <scheme val="none"/>
+      </font>
+      <alignment horizontal="left" vertical="top" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
   </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -971,16 +1017,18 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="Table1" displayName="Table1" ref="A1:L33" totalsRowShown="0">
-  <autoFilter ref="A1:L33" xr:uid="{00000000-0009-0000-0100-000001000000}"/>
-  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:K33">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="Table1" displayName="Table1" ref="A1:N33" totalsRowShown="0">
+  <autoFilter ref="A1:N33" xr:uid="{00000000-0009-0000-0100-000001000000}"/>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:M33">
     <sortCondition ref="A1:A33"/>
   </sortState>
-  <tableColumns count="12">
+  <tableColumns count="14">
     <tableColumn id="1" xr3:uid="{00000000-0010-0000-0000-000001000000}" name="ID"/>
     <tableColumn id="2" xr3:uid="{00000000-0010-0000-0000-000002000000}" name="Name"/>
     <tableColumn id="3" xr3:uid="{00000000-0010-0000-0000-000003000000}" name="Location Type List"/>
     <tableColumn id="4" xr3:uid="{00000000-0010-0000-0000-000004000000}" name="Geoname ID"/>
+    <tableColumn id="13" xr3:uid="{5C2EE668-4FB1-484C-B6F8-ADDBB38BAF5B}" name="Coordinates Latitude" dataDxfId="4"/>
+    <tableColumn id="14" xr3:uid="{081C0B36-7DF3-324C-BCFB-8E412BD2C9B7}" name="Coordinates Longitude" dataDxfId="3"/>
     <tableColumn id="5" xr3:uid="{00000000-0010-0000-0000-000005000000}" name="Image ID"/>
     <tableColumn id="12" xr3:uid="{2BD6E00F-E1B9-4940-B657-7C672A29756B}" name="Region ID" dataDxfId="2"/>
     <tableColumn id="6" xr3:uid="{00000000-0010-0000-0000-000006000000}" name="Description EN"/>
@@ -1170,23 +1218,24 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:L37"/>
+  <dimension ref="A1:N37"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="12.6640625" defaultRowHeight="18" x14ac:dyDescent="0.15"/>
   <cols>
     <col min="1" max="1" width="12.6640625" style="1" customWidth="1"/>
     <col min="2" max="2" width="39.6640625" style="1" customWidth="1"/>
     <col min="4" max="4" width="12.1640625" style="1" customWidth="1"/>
-    <col min="5" max="6" width="25.6640625" style="1" customWidth="1"/>
-    <col min="7" max="7" width="66.33203125" style="1" customWidth="1"/>
-    <col min="8" max="8" width="72.6640625" style="1" customWidth="1"/>
-    <col min="9" max="9" width="80" style="1" customWidth="1"/>
-    <col min="10" max="10" width="76.33203125" style="1" customWidth="1"/>
-    <col min="11" max="11" width="42.5" style="1" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="17.6640625" style="1" bestFit="1" customWidth="1"/>
-    <col min="13" max="16384" width="12.6640625" style="1"/>
+    <col min="5" max="6" width="24.83203125" style="1" customWidth="1"/>
+    <col min="7" max="8" width="25.6640625" style="1" customWidth="1"/>
+    <col min="9" max="9" width="66.33203125" style="1" customWidth="1"/>
+    <col min="10" max="10" width="72.6640625" style="1" customWidth="1"/>
+    <col min="11" max="11" width="80" style="1" customWidth="1"/>
+    <col min="12" max="12" width="76.33203125" style="1" customWidth="1"/>
+    <col min="13" max="13" width="42.5" style="1" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="17.6640625" style="1" bestFit="1" customWidth="1"/>
+    <col min="15" max="16384" width="12.6640625" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:12" s="3" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="1" spans="1:14" s="3" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
@@ -1200,31 +1249,37 @@
         <v>3</v>
       </c>
       <c r="E1" s="2" t="s">
+        <v>236</v>
+      </c>
+      <c r="F1" s="2" t="s">
+        <v>235</v>
+      </c>
+      <c r="G1" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="2" t="s">
+      <c r="H1" s="2" t="s">
         <v>232</v>
       </c>
-      <c r="G1" s="2" t="s">
+      <c r="I1" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="H1" s="2" t="s">
+      <c r="J1" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="I1" s="2" t="s">
+      <c r="K1" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="J1" s="2" t="s">
+      <c r="L1" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="K1" s="3" t="s">
+      <c r="M1" s="3" t="s">
         <v>9</v>
       </c>
-      <c r="L1" s="3" t="s">
+      <c r="N1" s="3" t="s">
         <v>229</v>
       </c>
     </row>
-    <row r="2" spans="1:12" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:14" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A2" s="4" t="s">
         <v>10</v>
       </c>
@@ -1235,25 +1290,27 @@
         <v>12</v>
       </c>
       <c r="D2" s="4"/>
-      <c r="E2" s="5"/>
-      <c r="F2" s="5"/>
-      <c r="G2" s="7" t="s">
+      <c r="E2" s="4"/>
+      <c r="F2" s="4"/>
+      <c r="G2" s="5"/>
+      <c r="H2" s="5"/>
+      <c r="I2" s="7" t="s">
         <v>13</v>
       </c>
-      <c r="H2" s="5" t="s">
+      <c r="J2" s="5" t="s">
         <v>14</v>
       </c>
-      <c r="I2" s="8" t="s">
+      <c r="K2" s="8" t="s">
         <v>15</v>
       </c>
-      <c r="J2" s="8" t="s">
+      <c r="L2" s="8" t="s">
         <v>16</v>
       </c>
-      <c r="K2" s="1" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="3" spans="1:12" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="M2" s="1" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="3" spans="1:14" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A3" s="4" t="s">
         <v>18</v>
       </c>
@@ -1264,27 +1321,29 @@
         <v>20</v>
       </c>
       <c r="D3" s="4"/>
-      <c r="E3" s="5" t="s">
+      <c r="E3" s="4"/>
+      <c r="F3" s="4"/>
+      <c r="G3" s="5" t="s">
         <v>21</v>
       </c>
-      <c r="F3" s="5"/>
-      <c r="G3" s="7" t="s">
+      <c r="H3" s="5"/>
+      <c r="I3" s="7" t="s">
         <v>22</v>
       </c>
-      <c r="H3" s="5" t="s">
+      <c r="J3" s="5" t="s">
         <v>23</v>
       </c>
-      <c r="I3" s="8" t="s">
+      <c r="K3" s="8" t="s">
         <v>24</v>
       </c>
-      <c r="J3" s="8" t="s">
+      <c r="L3" s="8" t="s">
         <v>25</v>
       </c>
-      <c r="K3" s="1" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="4" spans="1:12" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="M3" s="1" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="4" spans="1:14" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A4" s="4" t="s">
         <v>26</v>
       </c>
@@ -1295,27 +1354,29 @@
         <v>20</v>
       </c>
       <c r="D4" s="4"/>
-      <c r="E4" s="8" t="s">
+      <c r="E4" s="4"/>
+      <c r="F4" s="4"/>
+      <c r="G4" s="8" t="s">
         <v>28</v>
       </c>
-      <c r="F4" s="8"/>
-      <c r="G4" s="7" t="s">
+      <c r="H4" s="8"/>
+      <c r="I4" s="7" t="s">
         <v>29</v>
       </c>
-      <c r="H4" s="5" t="s">
+      <c r="J4" s="5" t="s">
         <v>30</v>
       </c>
-      <c r="I4" s="8" t="s">
+      <c r="K4" s="8" t="s">
         <v>31</v>
       </c>
-      <c r="J4" s="8" t="s">
+      <c r="L4" s="8" t="s">
         <v>32</v>
       </c>
-      <c r="K4" s="1" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="5" spans="1:12" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="M4" s="1" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="5" spans="1:14" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A5" s="4" t="s">
         <v>33</v>
       </c>
@@ -1326,29 +1387,31 @@
         <v>20</v>
       </c>
       <c r="D5" s="4"/>
-      <c r="E5" s="8" t="s">
+      <c r="E5" s="4"/>
+      <c r="F5" s="4"/>
+      <c r="G5" s="8" t="s">
         <v>35</v>
       </c>
-      <c r="F5" s="8" t="s">
+      <c r="H5" s="8" t="s">
         <v>234</v>
       </c>
-      <c r="G5" s="7" t="s">
+      <c r="I5" s="7" t="s">
         <v>36</v>
       </c>
-      <c r="H5" s="5" t="s">
+      <c r="J5" s="5" t="s">
         <v>37</v>
       </c>
-      <c r="I5" s="8" t="s">
+      <c r="K5" s="8" t="s">
         <v>38</v>
       </c>
-      <c r="J5" s="8" t="s">
+      <c r="L5" s="8" t="s">
         <v>39</v>
       </c>
-      <c r="K5" s="1" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="6" spans="1:12" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="M5" s="1" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="6" spans="1:14" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A6" s="4" t="s">
         <v>40</v>
       </c>
@@ -1359,25 +1422,27 @@
         <v>20</v>
       </c>
       <c r="D6" s="4"/>
-      <c r="E6" s="5"/>
-      <c r="F6" s="5"/>
-      <c r="G6" s="7" t="s">
+      <c r="E6" s="4"/>
+      <c r="F6" s="4"/>
+      <c r="G6" s="5"/>
+      <c r="H6" s="5"/>
+      <c r="I6" s="7" t="s">
         <v>42</v>
       </c>
-      <c r="H6" s="5" t="s">
+      <c r="J6" s="5" t="s">
         <v>43</v>
       </c>
-      <c r="I6" s="8" t="s">
+      <c r="K6" s="8" t="s">
         <v>44</v>
       </c>
-      <c r="J6" s="8" t="s">
+      <c r="L6" s="8" t="s">
         <v>45</v>
       </c>
-      <c r="K6" s="1" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="7" spans="1:12" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="M6" s="1" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="7" spans="1:14" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A7" s="4" t="s">
         <v>46</v>
       </c>
@@ -1388,25 +1453,27 @@
         <v>20</v>
       </c>
       <c r="D7" s="4"/>
-      <c r="E7" s="5"/>
-      <c r="F7" s="5"/>
-      <c r="G7" s="7" t="s">
+      <c r="E7" s="4"/>
+      <c r="F7" s="4"/>
+      <c r="G7" s="5"/>
+      <c r="H7" s="5"/>
+      <c r="I7" s="7" t="s">
         <v>48</v>
       </c>
-      <c r="H7" s="5" t="s">
+      <c r="J7" s="5" t="s">
         <v>49</v>
       </c>
-      <c r="I7" s="8" t="s">
+      <c r="K7" s="8" t="s">
         <v>50</v>
       </c>
-      <c r="J7" s="8" t="s">
+      <c r="L7" s="8" t="s">
         <v>51</v>
       </c>
-      <c r="K7" s="1" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="8" spans="1:12" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="M7" s="1" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="8" spans="1:14" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A8" s="4" t="s">
         <v>52</v>
       </c>
@@ -1417,27 +1484,29 @@
         <v>20</v>
       </c>
       <c r="D8" s="4"/>
-      <c r="E8" s="8" t="s">
+      <c r="E8" s="4"/>
+      <c r="F8" s="4"/>
+      <c r="G8" s="8" t="s">
         <v>54</v>
       </c>
-      <c r="F8" s="8"/>
-      <c r="G8" s="7" t="s">
+      <c r="H8" s="8"/>
+      <c r="I8" s="7" t="s">
         <v>55</v>
       </c>
-      <c r="H8" s="5" t="s">
+      <c r="J8" s="5" t="s">
         <v>56</v>
       </c>
-      <c r="I8" s="8" t="s">
+      <c r="K8" s="8" t="s">
         <v>57</v>
       </c>
-      <c r="J8" s="8" t="s">
+      <c r="L8" s="8" t="s">
         <v>58</v>
       </c>
-      <c r="K8" s="1" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="9" spans="1:12" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="M8" s="1" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="9" spans="1:14" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A9" s="4" t="s">
         <v>59</v>
       </c>
@@ -1448,27 +1517,29 @@
         <v>20</v>
       </c>
       <c r="D9" s="4"/>
-      <c r="E9" s="5" t="s">
+      <c r="E9" s="4"/>
+      <c r="F9" s="4"/>
+      <c r="G9" s="5" t="s">
         <v>61</v>
       </c>
-      <c r="F9" s="5"/>
-      <c r="G9" s="7" t="s">
+      <c r="H9" s="5"/>
+      <c r="I9" s="7" t="s">
         <v>62</v>
       </c>
-      <c r="H9" s="5" t="s">
+      <c r="J9" s="5" t="s">
         <v>63</v>
       </c>
-      <c r="I9" s="8" t="s">
+      <c r="K9" s="8" t="s">
         <v>64</v>
       </c>
-      <c r="J9" s="8" t="s">
+      <c r="L9" s="8" t="s">
         <v>65</v>
       </c>
-      <c r="K9" s="1" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="10" spans="1:12" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="M9" s="1" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="10" spans="1:14" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A10" s="4" t="s">
         <v>66</v>
       </c>
@@ -1481,28 +1552,34 @@
       <c r="D10" s="4">
         <v>2640729</v>
       </c>
-      <c r="E10" s="5"/>
-      <c r="F10" s="5"/>
-      <c r="G10" s="7" t="s">
+      <c r="E10" s="4">
+        <v>51.752220000000001</v>
+      </c>
+      <c r="F10" s="4">
+        <v>-1.25596</v>
+      </c>
+      <c r="G10" s="5"/>
+      <c r="H10" s="5"/>
+      <c r="I10" s="7" t="s">
         <v>68</v>
       </c>
-      <c r="H10" s="5" t="s">
+      <c r="J10" s="5" t="s">
         <v>69</v>
       </c>
-      <c r="I10" s="8" t="s">
+      <c r="K10" s="8" t="s">
         <v>70</v>
       </c>
-      <c r="J10" s="8" t="s">
+      <c r="L10" s="8" t="s">
         <v>71</v>
       </c>
-      <c r="K10" s="1" t="s">
-        <v>17</v>
-      </c>
-      <c r="L10" s="1" t="s">
+      <c r="M10" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="N10" s="1" t="s">
         <v>230</v>
       </c>
     </row>
-    <row r="11" spans="1:12" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:14" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A11" s="4" t="s">
         <v>72</v>
       </c>
@@ -1515,28 +1592,34 @@
       <c r="D11" s="4">
         <v>6269131</v>
       </c>
-      <c r="E11" s="5"/>
-      <c r="F11" s="5"/>
-      <c r="G11" s="7" t="s">
+      <c r="E11" s="4">
+        <v>52.160449999999997</v>
+      </c>
+      <c r="F11" s="4">
+        <v>-0.70311999999999997</v>
+      </c>
+      <c r="G11" s="5"/>
+      <c r="H11" s="5"/>
+      <c r="I11" s="7" t="s">
         <v>74</v>
       </c>
-      <c r="H11" s="5" t="s">
+      <c r="J11" s="5" t="s">
         <v>75</v>
       </c>
-      <c r="I11" s="8" t="s">
+      <c r="K11" s="8" t="s">
         <v>76</v>
       </c>
-      <c r="J11" s="8" t="s">
+      <c r="L11" s="8" t="s">
         <v>77</v>
       </c>
-      <c r="K11" s="1" t="s">
-        <v>17</v>
-      </c>
-      <c r="L11" s="1" t="s">
+      <c r="M11" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="N11" s="1" t="s">
         <v>231</v>
       </c>
     </row>
-    <row r="12" spans="1:12" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:14" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A12" s="4" t="s">
         <v>78</v>
       </c>
@@ -1547,27 +1630,29 @@
         <v>20</v>
       </c>
       <c r="D12" s="4"/>
-      <c r="E12" s="5" t="s">
+      <c r="E12" s="4"/>
+      <c r="F12" s="4"/>
+      <c r="G12" s="5" t="s">
         <v>80</v>
       </c>
-      <c r="F12" s="5"/>
-      <c r="G12" s="7" t="s">
+      <c r="H12" s="5"/>
+      <c r="I12" s="7" t="s">
         <v>81</v>
       </c>
-      <c r="H12" s="5" t="s">
+      <c r="J12" s="5" t="s">
         <v>82</v>
       </c>
-      <c r="I12" s="8" t="s">
+      <c r="K12" s="8" t="s">
         <v>83</v>
       </c>
-      <c r="J12" s="8" t="s">
+      <c r="L12" s="8" t="s">
         <v>84</v>
       </c>
-      <c r="K12" s="1" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="13" spans="1:12" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="M12" s="1" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="13" spans="1:14" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A13" s="4" t="s">
         <v>85</v>
       </c>
@@ -1578,27 +1663,29 @@
         <v>20</v>
       </c>
       <c r="D13" s="4"/>
-      <c r="E13" s="8" t="s">
+      <c r="E13" s="4"/>
+      <c r="F13" s="4"/>
+      <c r="G13" s="8" t="s">
         <v>87</v>
       </c>
-      <c r="F13" s="8"/>
-      <c r="G13" s="7" t="s">
+      <c r="H13" s="8"/>
+      <c r="I13" s="7" t="s">
         <v>88</v>
       </c>
-      <c r="H13" s="5" t="s">
+      <c r="J13" s="5" t="s">
         <v>89</v>
       </c>
-      <c r="I13" s="8" t="s">
+      <c r="K13" s="8" t="s">
         <v>90</v>
       </c>
-      <c r="J13" s="8" t="s">
+      <c r="L13" s="8" t="s">
         <v>91</v>
       </c>
-      <c r="K13" s="1" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="14" spans="1:12" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="M13" s="1" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="14" spans="1:14" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A14" s="4" t="s">
         <v>92</v>
       </c>
@@ -1609,27 +1696,29 @@
         <v>20</v>
       </c>
       <c r="D14" s="4"/>
-      <c r="E14" s="5" t="s">
+      <c r="E14" s="4"/>
+      <c r="F14" s="4"/>
+      <c r="G14" s="5" t="s">
         <v>94</v>
       </c>
-      <c r="F14" s="5"/>
-      <c r="G14" s="7" t="s">
+      <c r="H14" s="5"/>
+      <c r="I14" s="7" t="s">
         <v>95</v>
       </c>
-      <c r="H14" s="5" t="s">
+      <c r="J14" s="5" t="s">
         <v>96</v>
       </c>
-      <c r="I14" s="8" t="s">
+      <c r="K14" s="8" t="s">
         <v>97</v>
       </c>
-      <c r="J14" s="8" t="s">
+      <c r="L14" s="8" t="s">
         <v>98</v>
       </c>
-      <c r="K14" s="1" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="15" spans="1:12" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="M14" s="1" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="15" spans="1:14" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A15" s="4" t="s">
         <v>99</v>
       </c>
@@ -1640,27 +1729,29 @@
         <v>20</v>
       </c>
       <c r="D15" s="4"/>
-      <c r="E15" s="8" t="s">
+      <c r="E15" s="4"/>
+      <c r="F15" s="4"/>
+      <c r="G15" s="8" t="s">
         <v>101</v>
       </c>
-      <c r="F15" s="8"/>
-      <c r="G15" s="7" t="s">
+      <c r="H15" s="8"/>
+      <c r="I15" s="7" t="s">
         <v>102</v>
       </c>
-      <c r="H15" s="5" t="s">
+      <c r="J15" s="5" t="s">
         <v>103</v>
       </c>
-      <c r="I15" s="8" t="s">
+      <c r="K15" s="8" t="s">
         <v>104</v>
       </c>
-      <c r="J15" s="8" t="s">
+      <c r="L15" s="8" t="s">
         <v>105</v>
       </c>
-      <c r="K15" s="1" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="16" spans="1:12" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="M15" s="1" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="16" spans="1:14" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A16" s="4" t="s">
         <v>106</v>
       </c>
@@ -1671,25 +1762,27 @@
         <v>20</v>
       </c>
       <c r="D16" s="6"/>
-      <c r="E16" s="5"/>
-      <c r="F16" s="5"/>
-      <c r="G16" s="7" t="s">
+      <c r="E16" s="6"/>
+      <c r="F16" s="6"/>
+      <c r="G16" s="5"/>
+      <c r="H16" s="5"/>
+      <c r="I16" s="7" t="s">
         <v>108</v>
       </c>
-      <c r="H16" s="5" t="s">
+      <c r="J16" s="5" t="s">
         <v>109</v>
       </c>
-      <c r="I16" s="8" t="s">
+      <c r="K16" s="8" t="s">
         <v>110</v>
       </c>
-      <c r="J16" s="8" t="s">
+      <c r="L16" s="8" t="s">
         <v>111</v>
       </c>
-      <c r="K16" s="1" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="17" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="M16" s="1" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="17" spans="1:13" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A17" s="4" t="s">
         <v>112</v>
       </c>
@@ -1700,27 +1793,29 @@
         <v>20</v>
       </c>
       <c r="D17" s="6"/>
-      <c r="E17" s="8" t="s">
+      <c r="E17" s="6"/>
+      <c r="F17" s="6"/>
+      <c r="G17" s="8" t="s">
         <v>114</v>
       </c>
-      <c r="F17" s="8"/>
-      <c r="G17" s="7" t="s">
+      <c r="H17" s="8"/>
+      <c r="I17" s="7" t="s">
         <v>115</v>
       </c>
-      <c r="H17" s="5" t="s">
+      <c r="J17" s="5" t="s">
         <v>116</v>
       </c>
-      <c r="I17" s="8" t="s">
+      <c r="K17" s="8" t="s">
         <v>117</v>
       </c>
-      <c r="J17" s="8" t="s">
+      <c r="L17" s="8" t="s">
         <v>118</v>
       </c>
-      <c r="K17" s="1" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="18" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="M17" s="1" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="18" spans="1:13" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A18" s="4" t="s">
         <v>119</v>
       </c>
@@ -1731,27 +1826,29 @@
         <v>20</v>
       </c>
       <c r="D18" s="6"/>
-      <c r="E18" s="8" t="s">
+      <c r="E18" s="6"/>
+      <c r="F18" s="6"/>
+      <c r="G18" s="8" t="s">
         <v>121</v>
       </c>
-      <c r="F18" s="8"/>
-      <c r="G18" s="7" t="s">
+      <c r="H18" s="8"/>
+      <c r="I18" s="7" t="s">
         <v>122</v>
       </c>
-      <c r="H18" s="5" t="s">
+      <c r="J18" s="5" t="s">
         <v>123</v>
       </c>
-      <c r="I18" s="8" t="s">
+      <c r="K18" s="8" t="s">
         <v>124</v>
       </c>
-      <c r="J18" s="8" t="s">
+      <c r="L18" s="8" t="s">
         <v>125</v>
       </c>
-      <c r="K18" s="1" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="19" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="M18" s="1" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="19" spans="1:13" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A19" s="4" t="s">
         <v>126</v>
       </c>
@@ -1762,27 +1859,29 @@
         <v>20</v>
       </c>
       <c r="D19" s="6"/>
-      <c r="E19" s="8" t="s">
+      <c r="E19" s="6"/>
+      <c r="F19" s="6"/>
+      <c r="G19" s="8" t="s">
         <v>128</v>
       </c>
-      <c r="F19" s="8"/>
-      <c r="G19" s="7" t="s">
+      <c r="H19" s="8"/>
+      <c r="I19" s="7" t="s">
         <v>129</v>
       </c>
-      <c r="H19" s="5" t="s">
+      <c r="J19" s="5" t="s">
         <v>130</v>
       </c>
-      <c r="I19" s="8" t="s">
+      <c r="K19" s="8" t="s">
         <v>131</v>
       </c>
-      <c r="J19" s="8" t="s">
+      <c r="L19" s="8" t="s">
         <v>132</v>
       </c>
-      <c r="K19" s="1" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="20" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="M19" s="1" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="20" spans="1:13" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A20" s="4" t="s">
         <v>133</v>
       </c>
@@ -1793,27 +1892,29 @@
         <v>12</v>
       </c>
       <c r="D20" s="6"/>
-      <c r="E20" s="5" t="s">
+      <c r="E20" s="6"/>
+      <c r="F20" s="6"/>
+      <c r="G20" s="5" t="s">
         <v>135</v>
       </c>
-      <c r="F20" s="5"/>
-      <c r="G20" s="7" t="s">
+      <c r="H20" s="5"/>
+      <c r="I20" s="7" t="s">
         <v>136</v>
       </c>
-      <c r="H20" s="5" t="s">
+      <c r="J20" s="5" t="s">
         <v>137</v>
       </c>
-      <c r="I20" s="8" t="s">
+      <c r="K20" s="8" t="s">
         <v>138</v>
       </c>
-      <c r="J20" s="8" t="s">
+      <c r="L20" s="8" t="s">
         <v>139</v>
       </c>
-      <c r="K20" s="1" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="21" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="M20" s="1" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="21" spans="1:13" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A21" s="4" t="s">
         <v>140</v>
       </c>
@@ -1824,27 +1925,29 @@
         <v>20</v>
       </c>
       <c r="D21" s="6"/>
-      <c r="E21" s="5" t="s">
+      <c r="E21" s="6"/>
+      <c r="F21" s="6"/>
+      <c r="G21" s="5" t="s">
         <v>142</v>
       </c>
-      <c r="F21" s="5"/>
-      <c r="G21" s="7" t="s">
+      <c r="H21" s="5"/>
+      <c r="I21" s="7" t="s">
         <v>143</v>
       </c>
-      <c r="H21" s="5" t="s">
+      <c r="J21" s="5" t="s">
         <v>144</v>
       </c>
-      <c r="I21" s="8" t="s">
+      <c r="K21" s="8" t="s">
         <v>145</v>
       </c>
-      <c r="J21" s="8" t="s">
+      <c r="L21" s="8" t="s">
         <v>146</v>
       </c>
-      <c r="K21" s="1" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="22" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="M21" s="1" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="22" spans="1:13" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A22" s="4" t="s">
         <v>147</v>
       </c>
@@ -1855,29 +1958,31 @@
         <v>20</v>
       </c>
       <c r="D22" s="6"/>
-      <c r="E22" s="8" t="s">
+      <c r="E22" s="6"/>
+      <c r="F22" s="6"/>
+      <c r="G22" s="8" t="s">
         <v>149</v>
       </c>
-      <c r="F22" s="8" t="s">
+      <c r="H22" s="8" t="s">
         <v>233</v>
       </c>
-      <c r="G22" s="7" t="s">
+      <c r="I22" s="7" t="s">
         <v>150</v>
       </c>
-      <c r="H22" s="5" t="s">
+      <c r="J22" s="5" t="s">
         <v>151</v>
       </c>
-      <c r="I22" s="8" t="s">
+      <c r="K22" s="8" t="s">
         <v>152</v>
       </c>
-      <c r="J22" s="8" t="s">
+      <c r="L22" s="8" t="s">
         <v>153</v>
       </c>
-      <c r="K22" s="1" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="23" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="M22" s="1" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="23" spans="1:13" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A23" s="4" t="s">
         <v>154</v>
       </c>
@@ -1888,27 +1993,29 @@
         <v>20</v>
       </c>
       <c r="D23" s="6"/>
-      <c r="E23" s="5" t="s">
+      <c r="E23" s="6"/>
+      <c r="F23" s="6"/>
+      <c r="G23" s="5" t="s">
         <v>156</v>
       </c>
-      <c r="F23" s="5"/>
-      <c r="G23" s="7" t="s">
+      <c r="H23" s="5"/>
+      <c r="I23" s="7" t="s">
         <v>157</v>
       </c>
-      <c r="H23" s="5" t="s">
+      <c r="J23" s="5" t="s">
         <v>158</v>
       </c>
-      <c r="I23" s="8" t="s">
+      <c r="K23" s="8" t="s">
         <v>159</v>
       </c>
-      <c r="J23" s="8" t="s">
+      <c r="L23" s="8" t="s">
         <v>160</v>
       </c>
-      <c r="K23" s="1" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="24" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="M23" s="1" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="24" spans="1:13" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A24" s="4" t="s">
         <v>161</v>
       </c>
@@ -1919,27 +2026,29 @@
         <v>20</v>
       </c>
       <c r="D24" s="6"/>
-      <c r="E24" s="8" t="s">
+      <c r="E24" s="6"/>
+      <c r="F24" s="6"/>
+      <c r="G24" s="8" t="s">
         <v>163</v>
       </c>
-      <c r="F24" s="8"/>
-      <c r="G24" s="7" t="s">
+      <c r="H24" s="8"/>
+      <c r="I24" s="7" t="s">
         <v>164</v>
       </c>
-      <c r="H24" s="5" t="s">
+      <c r="J24" s="5" t="s">
         <v>165</v>
       </c>
-      <c r="I24" s="8" t="s">
+      <c r="K24" s="8" t="s">
         <v>166</v>
       </c>
-      <c r="J24" s="8" t="s">
+      <c r="L24" s="8" t="s">
         <v>167</v>
       </c>
-      <c r="K24" s="1" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="25" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="M24" s="1" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="25" spans="1:13" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A25" s="4" t="s">
         <v>168</v>
       </c>
@@ -1950,27 +2059,29 @@
         <v>20</v>
       </c>
       <c r="D25" s="6"/>
-      <c r="E25" s="5" t="s">
+      <c r="E25" s="6"/>
+      <c r="F25" s="6"/>
+      <c r="G25" s="5" t="s">
         <v>170</v>
       </c>
-      <c r="F25" s="5"/>
-      <c r="G25" s="7" t="s">
+      <c r="H25" s="5"/>
+      <c r="I25" s="7" t="s">
         <v>171</v>
       </c>
-      <c r="H25" s="5" t="s">
+      <c r="J25" s="5" t="s">
         <v>172</v>
       </c>
-      <c r="I25" s="8" t="s">
+      <c r="K25" s="8" t="s">
         <v>173</v>
       </c>
-      <c r="J25" s="8" t="s">
+      <c r="L25" s="8" t="s">
         <v>174</v>
       </c>
-      <c r="K25" s="1" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="26" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="M25" s="1" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="26" spans="1:13" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A26" s="4" t="s">
         <v>175</v>
       </c>
@@ -1981,27 +2092,29 @@
         <v>20</v>
       </c>
       <c r="D26" s="6"/>
-      <c r="E26" s="5" t="s">
+      <c r="E26" s="6"/>
+      <c r="F26" s="6"/>
+      <c r="G26" s="5" t="s">
         <v>177</v>
       </c>
-      <c r="F26" s="5"/>
-      <c r="G26" s="7" t="s">
+      <c r="H26" s="5"/>
+      <c r="I26" s="7" t="s">
         <v>178</v>
       </c>
-      <c r="H26" s="5" t="s">
+      <c r="J26" s="5" t="s">
         <v>179</v>
       </c>
-      <c r="I26" s="8" t="s">
+      <c r="K26" s="8" t="s">
         <v>180</v>
       </c>
-      <c r="J26" s="8" t="s">
+      <c r="L26" s="8" t="s">
         <v>181</v>
       </c>
-      <c r="K26" s="1" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="27" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="M26" s="1" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="27" spans="1:13" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A27" s="4" t="s">
         <v>182</v>
       </c>
@@ -2012,27 +2125,29 @@
         <v>20</v>
       </c>
       <c r="D27" s="6"/>
-      <c r="E27" s="8" t="s">
+      <c r="E27" s="6"/>
+      <c r="F27" s="6"/>
+      <c r="G27" s="8" t="s">
         <v>184</v>
       </c>
-      <c r="F27" s="8"/>
-      <c r="G27" s="7" t="s">
+      <c r="H27" s="8"/>
+      <c r="I27" s="7" t="s">
         <v>185</v>
       </c>
-      <c r="H27" s="5" t="s">
+      <c r="J27" s="5" t="s">
         <v>186</v>
       </c>
-      <c r="I27" s="8" t="s">
+      <c r="K27" s="8" t="s">
         <v>187</v>
       </c>
-      <c r="J27" s="8" t="s">
+      <c r="L27" s="8" t="s">
         <v>188</v>
       </c>
-      <c r="K27" s="1" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="28" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="M27" s="1" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="28" spans="1:13" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A28" s="4" t="s">
         <v>189</v>
       </c>
@@ -2043,27 +2158,29 @@
         <v>20</v>
       </c>
       <c r="D28" s="6"/>
-      <c r="E28" s="8" t="s">
+      <c r="E28" s="6"/>
+      <c r="F28" s="6"/>
+      <c r="G28" s="8" t="s">
         <v>191</v>
       </c>
-      <c r="F28" s="8"/>
-      <c r="G28" s="7" t="s">
+      <c r="H28" s="8"/>
+      <c r="I28" s="7" t="s">
         <v>192</v>
       </c>
-      <c r="H28" s="5" t="s">
+      <c r="J28" s="5" t="s">
         <v>193</v>
       </c>
-      <c r="I28" s="8" t="s">
+      <c r="K28" s="8" t="s">
         <v>194</v>
       </c>
-      <c r="J28" s="8" t="s">
+      <c r="L28" s="8" t="s">
         <v>195</v>
       </c>
-      <c r="K28" s="1" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="29" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="M28" s="1" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="29" spans="1:13" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A29" s="4" t="s">
         <v>196</v>
       </c>
@@ -2074,27 +2191,29 @@
         <v>20</v>
       </c>
       <c r="D29" s="6"/>
-      <c r="E29" s="5" t="s">
+      <c r="E29" s="6"/>
+      <c r="F29" s="6"/>
+      <c r="G29" s="5" t="s">
         <v>198</v>
       </c>
-      <c r="F29" s="5"/>
-      <c r="G29" s="7" t="s">
+      <c r="H29" s="5"/>
+      <c r="I29" s="7" t="s">
         <v>199</v>
       </c>
-      <c r="H29" s="5" t="s">
+      <c r="J29" s="5" t="s">
         <v>200</v>
       </c>
-      <c r="I29" s="8" t="s">
+      <c r="K29" s="8" t="s">
         <v>201</v>
       </c>
-      <c r="J29" s="8" t="s">
+      <c r="L29" s="8" t="s">
         <v>202</v>
       </c>
-      <c r="K29" s="1" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="30" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="M29" s="1" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="30" spans="1:13" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A30" s="4" t="s">
         <v>203</v>
       </c>
@@ -2105,27 +2224,29 @@
         <v>20</v>
       </c>
       <c r="D30" s="6"/>
-      <c r="E30" s="5" t="s">
+      <c r="E30" s="6"/>
+      <c r="F30" s="6"/>
+      <c r="G30" s="5" t="s">
         <v>205</v>
       </c>
-      <c r="F30" s="5"/>
-      <c r="G30" s="7" t="s">
+      <c r="H30" s="5"/>
+      <c r="I30" s="7" t="s">
         <v>206</v>
       </c>
-      <c r="H30" s="5" t="s">
+      <c r="J30" s="5" t="s">
         <v>207</v>
       </c>
-      <c r="I30" s="8" t="s">
+      <c r="K30" s="8" t="s">
         <v>208</v>
       </c>
-      <c r="J30" s="8" t="s">
+      <c r="L30" s="8" t="s">
         <v>209</v>
       </c>
-      <c r="K30" s="1" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="31" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="M30" s="1" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="31" spans="1:13" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A31" s="4" t="s">
         <v>210</v>
       </c>
@@ -2136,27 +2257,29 @@
         <v>20</v>
       </c>
       <c r="D31" s="6"/>
-      <c r="E31" s="5" t="s">
+      <c r="E31" s="6"/>
+      <c r="F31" s="6"/>
+      <c r="G31" s="5" t="s">
         <v>212</v>
       </c>
-      <c r="F31" s="5"/>
-      <c r="G31" s="7" t="s">
+      <c r="H31" s="5"/>
+      <c r="I31" s="7" t="s">
         <v>213</v>
       </c>
-      <c r="H31" s="5" t="s">
+      <c r="J31" s="5" t="s">
         <v>214</v>
       </c>
-      <c r="I31" s="8" t="s">
+      <c r="K31" s="8" t="s">
         <v>215</v>
       </c>
-      <c r="J31" s="8" t="s">
+      <c r="L31" s="8" t="s">
         <v>216</v>
       </c>
-      <c r="K31" s="1" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="32" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="M31" s="1" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="32" spans="1:13" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A32" s="4" t="s">
         <v>217</v>
       </c>
@@ -2167,25 +2290,27 @@
         <v>20</v>
       </c>
       <c r="D32" s="6"/>
-      <c r="E32" s="5"/>
-      <c r="F32" s="5"/>
-      <c r="G32" s="7" t="s">
+      <c r="E32" s="6"/>
+      <c r="F32" s="6"/>
+      <c r="G32" s="5"/>
+      <c r="H32" s="5"/>
+      <c r="I32" s="7" t="s">
         <v>219</v>
       </c>
-      <c r="H32" s="5" t="s">
+      <c r="J32" s="5" t="s">
         <v>220</v>
       </c>
-      <c r="I32" s="8" t="s">
+      <c r="K32" s="8" t="s">
         <v>221</v>
       </c>
-      <c r="J32" s="8" t="s">
+      <c r="L32" s="8" t="s">
         <v>222</v>
       </c>
-      <c r="K32" s="1" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="33" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="M32" s="1" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="33" spans="1:13" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A33" s="4" t="s">
         <v>223</v>
       </c>
@@ -2196,34 +2321,36 @@
         <v>20</v>
       </c>
       <c r="D33" s="6"/>
-      <c r="E33" s="5"/>
-      <c r="F33" s="5"/>
-      <c r="G33" s="7" t="s">
+      <c r="E33" s="6"/>
+      <c r="F33" s="6"/>
+      <c r="G33" s="5"/>
+      <c r="H33" s="5"/>
+      <c r="I33" s="7" t="s">
         <v>225</v>
       </c>
-      <c r="H33" s="5" t="s">
+      <c r="J33" s="5" t="s">
         <v>226</v>
       </c>
-      <c r="I33" s="8" t="s">
+      <c r="K33" s="8" t="s">
         <v>227</v>
       </c>
-      <c r="J33" s="8" t="s">
+      <c r="L33" s="8" t="s">
         <v>228</v>
       </c>
-      <c r="K33" s="1" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="34" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="M33" s="1" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="34" spans="1:13" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="B34" s="10"/>
     </row>
-    <row r="35" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="35" spans="1:13" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="B35" s="10"/>
     </row>
-    <row r="36" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="36" spans="1:13" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="B36" s="10"/>
     </row>
-    <row r="37" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="37" spans="1:13" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="B37" s="10"/>
     </row>
   </sheetData>

</xml_diff>